<commit_message>
Add and personalize leads for ReVision Energy and Sundial Solar
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V11"/>
+  <dimension ref="A1:V13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1400,19 +1400,188 @@
           <t>Google Maps</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
           <t>Co-founded in 2018 by Zachary Haithcock, Sean Carlson, and Scot Johnson. Headquartered in Exeter, NH. Provides turnkey residential and commercial solar PV installations across NH, Southern ME, and Northern MA. Named #1 Solar Company in Best of the 603 and Best of the Seacoast community choice awards (2023-2025). Direct contacts: zach@603solar.com and sean@603solar.com.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Solar Panel Company</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Brentwood, New Hampshire</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ReVisionEnergy</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/revisionenergy</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/revision-energy</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>https://www.revisionenergy.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>ReVision Energy</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Fortunat Mueller</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>(603) 679-1777</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>fortunat@revisionenergy.com</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>phil@revisionenergy.com</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>hello@revisionenergy.com</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>https://coldemail-dun.vercel.app/coldemail/ReVisionEnergy/index.html</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>Full-service 100% employee-owned solar contractor in Brentwood, NH founded in 2003 by Phil Coupe &amp; Fortunat Mueller. B-Corp certified with A+ BBB rating. 4.9 rating on Google (200+ reviews). Services include solar PV installation, Tesla Powerwall batteries, heat pumps, EV chargers. Runs in-house electrical apprenticeship school (RETC).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Solar Panel Company</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Concord, New Hampshire</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/SundialSolarNH</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/sundial-solar-nh</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>https://sundialsolarnh.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Sundial Solar</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Ryan Young</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>(603) 961-0045</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>ryan@sundialsolarnh.com</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>sales@sundialsolarnh.com</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>https://coldemail-dun.vercel.app/coldemail/SundialSolar/index.html</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>Full-service turnkey solar and geothermal contractor in Concord, NH active since 2015. Owned and managed by Ryan Young. Vetted EnergySage Approved installer using all in-house licensed crews instead of subcontractors. Services include solar PV installation, geothermal heating/cooling, battery backup, and heat pumps.</t>
         </is>
       </c>
     </row>

</xml_diff>